<commit_message>
Rebalancování: ceny, kurzy a datum ocenění v Excelu nepovinné, bez posuvníku při načítání
Šablona už ceny, kurzy ani datum ocenění nemá – doplní se z denních tržních dat.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NYgWYvTs4GD6m8QWa978gy
</commit_message>
<xml_diff>
--- a/rebalancing/sablona.xlsx
+++ b/rebalancing/sablona.xlsx
@@ -9,11 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Čti mě" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrumenty" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kurzy" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klienti" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pozice" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hotovost" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash flow" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klienti" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pozice" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hotovost" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash flow" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,10 +79,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -180,6 +179,11 @@
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>Ticker musí odpovídat sloupcům „Cíl … %“ v listu Klienti. Denní tržní ceny se stahují pro VWCE, AVWS, EUNA a IGLN.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Nevyplňuje se – cena se stáhne automaticky. Vyplňte jen u ETF, pro které tržní data nejsou (spolu se sloupcem Měna).</t>
       </text>
     </comment>
   </commentList>
@@ -510,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -524,76 +528,69 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Ocenění k datu: 29. 10. 2026</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr"/>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Jak vyplnit</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Jak vyplnit</t>
+          <t>1. Šedé kurzívou psané řádky jsou vzor – přepište je vlastními údaji nebo smažte.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>1. Šedé kurzívou psané řádky jsou vzor – přepište je vlastními údaji nebo smažte.</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2. Názvy listů a záhlaví sloupců neměňte, nástroj podle nich data čte.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2. Názvy listů a záhlaví sloupců neměňte, nástroj podle nich data čte.</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>3. Ceny ETF, kurzy měn ani datum ocenění se nevyplňují – nástroj je stáhne automaticky (závěrečné ceny ETF a kurzy ČNB z posledního obchodního dne). List Instrumenty je jen přehled; cenu a měnu do něj doplňte jen u ETF, pro které tržní data nejsou.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>3. Instrumenty: všechny ETF, které klienti drží nebo mají v cílech. Ceny a kurzy se při tržním ocenění doplní automaticky, vyplněné ale být musí (stačí poslední známé).</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>4. Klienti: cílové váhy v % celkového majetku včetně hotovosti, součet musí být 100. Daňový režim FO = fyzická osoba, s.r.o. = právnická osoba.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>4. Klienti: cílové váhy v % celkového majetku včetně hotovosti, součet musí být 100. Daňový režim FO = fyzická osoba, s.r.o. = právnická osoba.</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>5. Pozice: každý nákup zvlášť (kvůli časovému testu a FIFO) – datum nákupu, počet kusů a cena v měně instrumentu.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>5. Pozice: každý nákup zvlášť (kvůli časovému testu a FIFO) – datum nákupu, počet kusů a cena v měně instrumentu.</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>6. Hotovost: zůstatky podle měny. Cash flow: plánované vklady (kladné) a výběry (záporné) v CZK.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>6. Hotovost: zůstatky podle měny. Cash flow: plánované vklady (kladné) a výběry (záporné) v CZK.</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>7. Pozice a hotovost vyplňte podle aktuálního výpisu od brokera. Vklady a výběry, které už proběhly, patří do hotovosti, ne do Cash flow.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>7. Řádek „Ocenění k datu“ výše je datum, ke kterému platí pozice a hotovost. Při tržním ocenění se ceny vezmou k poslednímu obchodnímu dni.</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Soubor se nikam neodesílá – zpracuje se jen ve vašem prohlížeči.</t>
         </is>
@@ -679,9 +676,7 @@
           <t>Akcie (globální)</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n">
-        <v>142.5</v>
-      </c>
+      <c r="F2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -709,9 +704,7 @@
           <t>Akcie (small cap value)</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n">
-        <v>12.6</v>
-      </c>
+      <c r="F3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -739,9 +732,7 @@
           <t>Dluhopisy</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n">
-        <v>4.62</v>
-      </c>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -769,9 +760,7 @@
           <t>Zlato</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
-        <v>78.40000000000001</v>
-      </c>
+      <c r="F5" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -780,56 +769,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Měnový pár</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Kurz (CZK za 1 jednotku)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>EUR/CZK</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n">
-        <v>24.3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>USD/CZK</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -944,7 +883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2508,7 +2447,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2564,7 +2503,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Rebalancování: ceny ETF podle ISIN (denní seznam + Cloudflare Worker), ETF bez ceny jen u dotčených klientů
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NYgWYvTs4GD6m8QWa978gy
</commit_message>
<xml_diff>
--- a/rebalancing/sablona.xlsx
+++ b/rebalancing/sablona.xlsx
@@ -178,12 +178,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Ticker musí odpovídat sloupcům „Cíl … %“ v listu Klienti. Denní tržní ceny se stahují pro VWCE, AVWS, EUNA a IGLN.</t>
+        <t>Ticker je jen váš název ETF – musí odpovídat sloupcům „Cíl … %“ v listu Klienti a listu Pozice.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>ISIN fondu (12 znaků, např. IE00B5BMR087). Podle něj se automaticky dohledá aktuální cena.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Měna, ve které jsou nákupní ceny v listu Pozice (EUR, USD, GBP, CHF). Tržní cena se do ní přepočte kurzem ČNB.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Nevyplňuje se – cena se stáhne automaticky. Vyplňte jen u ETF, pro které tržní data nejsou (spolu se sloupcem Měna).</t>
+        <t>Nevyplňuje se – cena se dohledá podle ISIN. Vyplňte jen, když ji nástroj nenajde.</t>
       </text>
     </comment>
   </commentList>
@@ -514,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -554,43 +564,57 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Ceny ETF, kurzy měn ani datum ocenění se nevyplňují – nástroj je stáhne automaticky (závěrečné ceny ETF a kurzy ČNB z posledního obchodního dne). List Instrumenty je jen přehled; cenu a měnu do něj doplňte jen u ETF, pro které tržní data nejsou.</t>
+          <t>3. Ceny ETF, kurzy měn ani datum ocenění se nevyplňují – nástroj je stáhne automaticky (závěrečné ceny a kurzy ČNB z posledního obchodního dne).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. Klienti: cílové váhy v % celkového majetku včetně hotovosti, součet musí být 100. Daňový režim FO = fyzická osoba, s.r.o. = právnická osoba.</t>
+          <t xml:space="preserve">   V listu Instrumenty uveďte u každého ETF ISIN – podle něj se dohledá aktuální cena, i u fondů mimo vzor. Měna = měna, ve které jsou nákupní ceny v listu Pozice.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5. Pozice: každý nákup zvlášť (kvůli časovému testu a FIFO) – datum nákupu, počet kusů a cena v měně instrumentu.</t>
+          <t xml:space="preserve">   Cenu vyplňte jen tehdy, když ji nástroj podle ISIN nenajde (ohlásí to).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>6. Hotovost: zůstatky podle měny. Cash flow: plánované vklady (kladné) a výběry (záporné) v CZK.</t>
+          <t>4. Klienti: cílové váhy v % celkového majetku včetně hotovosti, součet musí být 100. Daňový režim FO = fyzická osoba, s.r.o. = právnická osoba.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>5. Pozice: každý nákup zvlášť (kvůli časovému testu a FIFO) – datum nákupu, počet kusů a cena v měně instrumentu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>6. Hotovost: zůstatky podle měny. Cash flow: plánované vklady (kladné) a výběry (záporné) v CZK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>7. Pozice a hotovost vyplňte podle aktuálního výpisu od brokera. Vklady a výběry, které už proběhly, patří do hotovosti, ne do Cash flow.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Soubor se nikam neodesílá – zpracuje se jen ve vašem prohlížeči.</t>
         </is>

</xml_diff>